<commit_message>
Testcases updated and enhanced
</commit_message>
<xml_diff>
--- a/TestData/UserDetails.xlsx
+++ b/TestData/UserDetails.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RestAssurred\PetStoreAutomation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD2058F1-9631-478C-BE43-89CEA0881CB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C430060-A785-4EB9-B517-13DAFC859AB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E21C8D07-366E-4020-A7A3-5816D9F3417C}"/>
+    <workbookView xWindow="2652" yWindow="2652" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{E21C8D07-366E-4020-A7A3-5816D9F3417C}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="UserDetails" sheetId="1" r:id="rId1"/>
+    <sheet name="PetDetails" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="55">
   <si>
     <t>UserId</t>
   </si>
@@ -127,6 +128,78 @@
   </si>
   <si>
     <t>test@654</t>
+  </si>
+  <si>
+    <t>PetId</t>
+  </si>
+  <si>
+    <t>CategoryId</t>
+  </si>
+  <si>
+    <t>CategoryName</t>
+  </si>
+  <si>
+    <t>PetName</t>
+  </si>
+  <si>
+    <t>PetPhotoUrls</t>
+  </si>
+  <si>
+    <t>TagId</t>
+  </si>
+  <si>
+    <t>TagName</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>https://petweb.com/photo/doggie1.jpg,https://petweb.com/photo/doggie2.jpg</t>
+  </si>
+  <si>
+    <t>Available</t>
+  </si>
+  <si>
+    <t>Dog</t>
+  </si>
+  <si>
+    <t>qwerty</t>
+  </si>
+  <si>
+    <t>Cat</t>
+  </si>
+  <si>
+    <t>https://petweb.com/photo/cattie1.jpg,https://petweb.com/photo/cattie2.jpg</t>
+  </si>
+  <si>
+    <t>asdf</t>
+  </si>
+  <si>
+    <t>Doggie2</t>
+  </si>
+  <si>
+    <t>Doggie1</t>
+  </si>
+  <si>
+    <t>zxcvb</t>
+  </si>
+  <si>
+    <t>NotAvailable</t>
+  </si>
+  <si>
+    <t>Cattie2</t>
+  </si>
+  <si>
+    <t>etrrtry</t>
+  </si>
+  <si>
+    <t>https://petweb.com/photo/cattie3.jpg,https://petweb.com/photo/cattie4.jpg</t>
+  </si>
+  <si>
+    <t>https://petweb.com/photo/doggie3.jpg,https://petweb.com/photo/doggie4.jpg</t>
+  </si>
+  <si>
+    <t>Cattie1</t>
   </si>
 </sst>
 </file>
@@ -186,7 +259,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -196,6 +269,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -676,4 +752,157 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A68740FA-5394-44B7-B773-8F1F192E2198}">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.109375" customWidth="1"/>
+    <col min="2" max="2" width="12.21875" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" customWidth="1"/>
+    <col min="5" max="5" width="46.88671875" customWidth="1"/>
+    <col min="8" max="8" width="20.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>11011</v>
+      </c>
+      <c r="B2" s="1">
+        <v>11122</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" s="1">
+        <v>123</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>11022</v>
+      </c>
+      <c r="B3" s="1">
+        <v>11133</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" s="1">
+        <v>123</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>11033</v>
+      </c>
+      <c r="B4" s="1">
+        <v>11122</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F4" s="1">
+        <v>234</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>11044</v>
+      </c>
+      <c r="B5" s="1">
+        <v>11133</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F5" s="1">
+        <v>456</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{2F0446A1-98EA-4BC9-BC05-F982CD7E5549}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{BEC69449-2C9F-420A-8E22-301D2D77B1E7}"/>
+    <hyperlink ref="E4" r:id="rId3" xr:uid="{45991E3B-FE5B-4482-8556-06A3586B50FA}"/>
+    <hyperlink ref="E5" r:id="rId4" xr:uid="{4C532586-137E-400D-B1E2-8320F1E569F9}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>